<commit_message>
Intro as a panel with a close button; hero proof points and aligned 'three/fourth' rows; spreadsheets and slides, not vendor names
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/media/exports/services-sample-statements.xlsx
+++ b/media/exports/services-sample-statements.xlsx
@@ -1052,7 +1052,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 10:07am</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:30pm</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1355,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Advisory Pty Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 services-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 10:07am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 services-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:30pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -1442,7 +1442,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 10:07am</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:30pm</t>
         </is>
       </c>
     </row>
@@ -2059,7 +2059,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Advisory Pty Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 services-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 10:07am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 services-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:30pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2100,7 +2100,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 10:07am</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:30pm</t>
         </is>
       </c>
     </row>
@@ -2454,7 +2454,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Advisory Pty Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 services-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 10:07am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 services-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:30pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2495,7 +2495,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 10:07am</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:30pm</t>
         </is>
       </c>
     </row>
@@ -2883,7 +2883,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Advisory Pty Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 services-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 10:07am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 services-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:30pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -2930,7 +2930,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 10:07am</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:30pm</t>
         </is>
       </c>
     </row>
@@ -3813,7 +3813,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Advisory Pty Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 services-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 10:07am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 services-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:30pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -3858,7 +3858,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 10:07am</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:30pm</t>
         </is>
       </c>
     </row>
@@ -5105,7 +5105,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Advisory Pty Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 services-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 10:07am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 services-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:30pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>
@@ -5152,7 +5152,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 10:07am</t>
+          <t>Data status: Sep 2026 locked · Aug 2026 locked · Oct 2026 incomplete (data retrieved 2pm, Tue 6 Oct 2026) · Generated 8 Oct 2026, 9:30pm</t>
         </is>
       </c>
     </row>
@@ -5252,7 +5252,7 @@
       </c>
       <c r="B14" s="32" t="inlineStr">
         <is>
-          <t>10 (every one is in the Excel download and CSV)</t>
+          <t>10 (every one is in the spreadsheet download and CSV)</t>
         </is>
       </c>
     </row>
@@ -5469,7 +5469,7 @@
   <pageSetup orientation="landscape" paperSize="9" fitToHeight="0" fitToWidth="1"/>
   <headerFooter>
     <oddHeader>&amp;L&amp;"Roboto,Regular"&amp;8 Sample Advisory Pty Ltd&amp;R&amp;"Roboto,Regular"&amp;8 &amp;A</oddHeader>
-    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 services-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 10:07am&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
+    <oddFooter>&amp;L&amp;"Roboto,Regular"&amp;8 services-sample-statements.xlsx&amp;C&amp;"Roboto,Regular"&amp;8 Data retrieved 2pm, Tue 6 Oct 2026 · Generated 8 Oct 2026, 9:30pm&amp;R&amp;"Roboto,Regular"&amp;8 Page &amp;P of &amp;N</oddFooter>
     <evenHeader/>
     <evenFooter/>
     <firstHeader/>

</xml_diff>